<commit_message>
add  deberta base long
</commit_message>
<xml_diff>
--- a/comparison_table.xlsx
+++ b/comparison_table.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\tesis nli\contract-nli-increased\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40175DA9-3C38-45F6-A07E-7B9AA8C1ABF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11940" yWindow="1560" windowWidth="12885" windowHeight="13305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Model</t>
   </si>
@@ -35,6 +29,9 @@
   </si>
   <si>
     <t>Accuracy</t>
+  </si>
+  <si>
+    <t>deberta-base-long-nli.json</t>
   </si>
   <si>
     <t>deberta-small-long-nli.json</t>
@@ -46,8 +43,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,11 +102,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -117,21 +115,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -169,7 +159,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -203,7 +193,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -238,10 +227,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,14 +402,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -438,38 +423,55 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2">
-        <v>0.73164158632776444</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.72999035679845714</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.72992081369081352</v>
-      </c>
-      <c r="E2" s="2">
-        <v>0.72999035679845714</v>
+      <c r="B2" s="3">
+        <v>0.7389875046264152</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.7328833172613307</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0.7352495275195864</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.7328833172613307</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2">
-        <v>0.73436892365658346</v>
-      </c>
-      <c r="C3">
-        <v>0.72516875602700093</v>
-      </c>
-      <c r="D3">
-        <v>0.72839453038210089</v>
-      </c>
-      <c r="E3">
-        <v>0.72516875602700093</v>
+        <v>0.7316415863277644</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.7299903567984571</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.7299208136908135</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0.7299903567984571</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.7343689236565835</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.7251687560270009</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.7283945303821009</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.7251687560270009</v>
       </c>
     </row>
   </sheetData>

</xml_diff>